<commit_message>
upd fix error form e-invoice
</commit_message>
<xml_diff>
--- a/resources/report/60/95/rpt_6095170_1.xlsx
+++ b/resources/report/60/95/rpt_6095170_1.xlsx
@@ -92,9 +92,6 @@
     <t>Địa chỉ</t>
   </si>
   <si>
-    <t>SEQ</t>
-  </si>
-  <si>
     <t>FORM_NO</t>
   </si>
   <si>
@@ -137,10 +134,13 @@
     <t>ADDR</t>
   </si>
   <si>
-    <t>CANCEL_BY</t>
-  </si>
-  <si>
     <t>REMARK</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>ADJ_BY</t>
   </si>
 </sst>
 </file>
@@ -340,91 +340,91 @@
   </cellStyleXfs>
   <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -713,306 +713,312 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="2" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:17" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="29"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="29"/>
+      <c r="Q5" s="29"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="7"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="26"/>
+      <c r="Q6" s="26"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11"/>
+      <c r="O7" s="11"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10" t="s">
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="11" t="s">
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="Q8" s="12" t="s">
+      <c r="Q8" s="19" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="13"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="14" t="s">
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="17" t="s">
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="M9" s="18"/>
-      <c r="N9" s="18"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="12"/>
+      <c r="M9" s="24"/>
+      <c r="N9" s="24"/>
+      <c r="O9" s="25"/>
+      <c r="P9" s="17"/>
+      <c r="Q9" s="19"/>
     </row>
     <row r="10" spans="1:17" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
-      <c r="B10" s="22" t="s">
+      <c r="A10" s="14"/>
+      <c r="B10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="G10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="22" t="s">
+      <c r="H10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="22" t="s">
+      <c r="I10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J10" s="22" t="s">
+      <c r="J10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K10" s="22" t="s">
+      <c r="K10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="L10" s="23" t="s">
+      <c r="L10" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="M10" s="23" t="s">
+      <c r="M10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="N10" s="23" t="s">
+      <c r="N10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="O10" s="23" t="s">
+      <c r="O10" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="12"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="19"/>
     </row>
     <row r="11" spans="1:17" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="C11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="D11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="E11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="F11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="27" t="s">
+      <c r="G11" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="26" t="s">
+      <c r="H11" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="26" t="s">
+      <c r="I11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="I11" s="26" t="s">
+      <c r="J11" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="J11" s="26" t="s">
+      <c r="K11" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="K11" s="27" t="s">
+      <c r="L11" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="L11" s="28" t="s">
+      <c r="M11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="M11" s="29" t="s">
+      <c r="N11" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="N11" s="29" t="s">
+      <c r="O11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="O11" s="29" t="s">
+      <c r="P11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q11" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="P11" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q11" s="26" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A6:Q6"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A5:Q5"/>
     <mergeCell ref="A7:Q7"/>
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="B8:F9"/>
@@ -1021,13 +1027,8 @@
     <mergeCell ref="Q8:Q10"/>
     <mergeCell ref="G9:K9"/>
     <mergeCell ref="L9:O9"/>
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A5:Q5"/>
-    <mergeCell ref="A6:Q6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>